<commit_message>
some markup from tiago on pyrate old vs. new binning, pred importance for new interpolation method on model 9
</commit_message>
<xml_diff>
--- a/pyrate_features_binning/model_3_syn_new_pyrate_features.xlsx
+++ b/pyrate_features_binning/model_3_syn_new_pyrate_features.xlsx
@@ -8,15 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\pt_diversity_rates\pyrate_features_binning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BCE7063-F607-442F-A326-7828AEBC354E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BEB8A17-F107-4386-AD5C-7DBC6268D242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60060" yWindow="270" windowWidth="20880" windowHeight="9135" xr2:uid="{DD87EB3A-CD3F-4F95-9661-756DC8706995}"/>
+    <workbookView xWindow="57705" yWindow="645" windowWidth="22950" windowHeight="12195" xr2:uid="{DD87EB3A-CD3F-4F95-9661-756DC8706995}"/>
   </bookViews>
   <sheets>
     <sheet name="new_pyrate_features" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
   <si>
     <t>mat_z_trans</t>
   </si>
@@ -52,6 +63,48 @@
   </si>
   <si>
     <t>Time</t>
+  </si>
+  <si>
+    <t>Rhaetian</t>
+  </si>
+  <si>
+    <t>Sakmarian</t>
+  </si>
+  <si>
+    <t>Artinskian</t>
+  </si>
+  <si>
+    <t>Asselian</t>
+  </si>
+  <si>
+    <t>stage</t>
+  </si>
+  <si>
+    <t>Kungurian</t>
+  </si>
+  <si>
+    <t>Roadian</t>
+  </si>
+  <si>
+    <t>Wordian</t>
+  </si>
+  <si>
+    <t>Capit</t>
+  </si>
+  <si>
+    <t>Road+Word</t>
+  </si>
+  <si>
+    <t>Lopingian</t>
+  </si>
+  <si>
+    <t>Wuch</t>
+  </si>
+  <si>
+    <t>Chang</t>
+  </si>
+  <si>
+    <t>Time_stage_end_input</t>
   </si>
 </sst>
 </file>
@@ -194,7 +247,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -377,6 +430,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -541,10 +600,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -920,7 +980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F33D504-9697-4EF9-BBE2-34FFA7F3B0C2}">
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="7" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -928,9 +988,11 @@
     <col min="12" max="12" width="14.19921875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.9296875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.59765625" customWidth="1"/>
+    <col min="18" max="18" width="13.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
       <c r="G1" t="s">
         <v>0</v>
       </c>
@@ -958,8 +1020,20 @@
       <c r="P1" t="s">
         <v>8</v>
       </c>
+      <c r="Q1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" t="s">
+        <v>7</v>
+      </c>
+      <c r="T1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1009,8 +1083,20 @@
         <f>174.5+O2</f>
         <v>293.69637298583899</v>
       </c>
+      <c r="Q2" t="s">
+        <v>10</v>
+      </c>
+      <c r="R2">
+        <v>293.52</v>
+      </c>
+      <c r="S2">
+        <v>-0.94344203948899896</v>
+      </c>
+      <c r="T2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1060,8 +1146,20 @@
         <f t="shared" ref="P3:P14" si="0">174.5+O3</f>
         <v>286.30000305175702</v>
       </c>
+      <c r="Q3" t="s">
+        <v>11</v>
+      </c>
+      <c r="R3">
+        <v>290.10000000000002</v>
+      </c>
+      <c r="S3">
+        <v>-0.135395184672056</v>
+      </c>
+      <c r="T3" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1111,8 +1209,20 @@
         <f t="shared" si="0"/>
         <v>278.44999694824202</v>
       </c>
+      <c r="Q4" t="s">
+        <v>14</v>
+      </c>
+      <c r="R4">
+        <v>283.5</v>
+      </c>
+      <c r="S4">
+        <v>0.95395715690469796</v>
+      </c>
+      <c r="T4" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1152,7 +1262,7 @@
       <c r="M5" s="1">
         <v>0.80949175357818604</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="3">
         <v>-0.403737783432006</v>
       </c>
       <c r="O5" s="1">
@@ -1162,8 +1272,20 @@
         <f t="shared" si="0"/>
         <v>268.84999847412098</v>
       </c>
+      <c r="Q5" t="s">
+        <v>18</v>
+      </c>
+      <c r="R5">
+        <v>272.95</v>
+      </c>
+      <c r="S5">
+        <v>-9.6334319592016895E-2</v>
+      </c>
+      <c r="T5" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1213,8 +1335,20 @@
         <f t="shared" si="0"/>
         <v>261.40000152587891</v>
       </c>
+      <c r="Q6" t="s">
+        <v>17</v>
+      </c>
+      <c r="R6">
+        <v>268.8</v>
+      </c>
+      <c r="S6">
+        <v>-0.49210833709615998</v>
+      </c>
+      <c r="T6" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1254,7 +1388,7 @@
       <c r="M7" s="1">
         <v>0.14476403594017001</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="3">
         <v>0.29276031255722001</v>
       </c>
       <c r="O7" s="1">
@@ -1264,8 +1398,20 @@
         <f t="shared" si="0"/>
         <v>255.25</v>
       </c>
+      <c r="Q7" t="s">
+        <v>19</v>
+      </c>
+      <c r="R7">
+        <v>265.10000000000002</v>
+      </c>
+      <c r="S7">
+        <v>-0.62277071678001805</v>
+      </c>
+      <c r="T7" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1315,8 +1461,17 @@
         <f t="shared" si="0"/>
         <v>248.84999847412098</v>
       </c>
+      <c r="R8">
+        <v>259.10000000000002</v>
+      </c>
+      <c r="S8">
+        <v>0.71133556211286197</v>
+      </c>
+      <c r="T8" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1366,8 +1521,17 @@
         <f t="shared" si="0"/>
         <v>243.84999847412098</v>
       </c>
+      <c r="R9">
+        <v>254.14</v>
+      </c>
+      <c r="S9">
+        <v>-0.12581492327281199</v>
+      </c>
+      <c r="T9" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1417,8 +1581,17 @@
         <f t="shared" si="0"/>
         <v>239</v>
       </c>
+      <c r="R10">
+        <v>251.90199999999999</v>
+      </c>
+      <c r="S10">
+        <v>-0.88112743681619099</v>
+      </c>
+      <c r="T10" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1468,8 +1641,14 @@
         <f t="shared" si="0"/>
         <v>231.5</v>
       </c>
+      <c r="R11">
+        <v>251.2</v>
+      </c>
+      <c r="S11">
+        <v>-1.18038656898602E-2</v>
+      </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1519,8 +1698,14 @@
         <f t="shared" si="0"/>
         <v>221.5</v>
       </c>
+      <c r="R12">
+        <v>247.2</v>
+      </c>
+      <c r="S12">
+        <v>-0.59531514265798402</v>
+      </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1570,8 +1755,14 @@
         <f t="shared" si="0"/>
         <v>212</v>
       </c>
+      <c r="R13">
+        <v>242</v>
+      </c>
+      <c r="S13">
+        <v>-0.58085573967703197</v>
+      </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>-0.29742455482482899</v>
       </c>
@@ -1620,6 +1811,39 @@
       <c r="P14">
         <f t="shared" si="0"/>
         <v>191</v>
+      </c>
+      <c r="R14">
+        <v>237</v>
+      </c>
+      <c r="S14">
+        <v>-0.26759464512162301</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="R15">
+        <v>227</v>
+      </c>
+      <c r="S15">
+        <v>0.66131645771053804</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="R16">
+        <v>208.5</v>
+      </c>
+      <c r="S16">
+        <v>-0.79955166023046298</v>
+      </c>
+    </row>
+    <row r="17" spans="18:20" x14ac:dyDescent="0.45">
+      <c r="R17">
+        <v>201.3</v>
+      </c>
+      <c r="S17">
+        <v>3.2255048343671202</v>
+      </c>
+      <c r="T17" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>